<commit_message>
feat(tasks): implement ownership scoping, TASK-M10 project assignment, and dependency surfacing
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$G$303</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$G$308</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Florin - my actions'!$A$1:$D$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary'!$A$1:$B$36</definedName>
   </definedNames>
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -171,6 +171,7 @@
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G303"/>
+  <dimension ref="A1:G308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9514,9 +9515,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E266" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E266" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F266" s="11" t="inlineStr">
@@ -9526,7 +9527,7 @@
       </c>
       <c r="G266" s="11" t="inlineStr">
         <is>
-          <t>Do first, no deps</t>
+          <t>0648d7e</t>
         </is>
       </c>
     </row>
@@ -9621,9 +9622,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E269" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E269" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F269" s="11" t="inlineStr">
@@ -9631,7 +9632,11 @@
           <t>coder-directive-doc-archive.md</t>
         </is>
       </c>
-      <c r="G269" s="11" t="inlineStr"/>
+      <c r="G269" s="11" t="inlineStr">
+        <is>
+          <t>0648d7e</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="11" t="inlineStr">
@@ -9654,9 +9659,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="E270" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E270" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F270" s="11" t="inlineStr">
@@ -9666,7 +9671,7 @@
       </c>
       <c r="G270" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-09-12 — ships with DOC-ARCH-1, no R4 dependency</t>
+          <t>c529202</t>
         </is>
       </c>
     </row>
@@ -9761,9 +9766,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E273" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E273" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F273" s="11" t="inlineStr">
@@ -9773,7 +9778,7 @@
       </c>
       <c r="G273" s="11" t="inlineStr">
         <is>
-          <t>Blocks DOC-ARCH-1/5</t>
+          <t>e070a6f</t>
         </is>
       </c>
     </row>
@@ -9872,9 +9877,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E276" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E276" s="20" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F276" s="11" t="inlineStr">
@@ -9882,7 +9887,11 @@
           <t>coder-directive-tasks-part-a.md</t>
         </is>
       </c>
-      <c r="G276" s="11" t="inlineStr"/>
+      <c r="G276" s="11" t="inlineStr">
+        <is>
+          <t>260e29d — ownership filter + opt-* status still to correct</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="11" t="inlineStr">
@@ -9971,9 +9980,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E279" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E279" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F279" s="11" t="inlineStr">
@@ -9981,7 +9990,11 @@
           <t>coder-directive-tasks-part-a.md</t>
         </is>
       </c>
-      <c r="G279" s="11" t="inlineStr"/>
+      <c r="G279" s="11" t="inlineStr">
+        <is>
+          <t>260e29d</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="11" t="inlineStr">
@@ -10004,9 +10017,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="E280" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E280" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F280" s="11" t="inlineStr">
@@ -10014,7 +10027,11 @@
           <t>coder-directive-tasks-part-a.md</t>
         </is>
       </c>
-      <c r="G280" s="11" t="inlineStr"/>
+      <c r="G280" s="11" t="inlineStr">
+        <is>
+          <t>260e29d</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="11" t="inlineStr">
@@ -10037,9 +10054,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="E281" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E281" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F281" s="11" t="inlineStr">
@@ -10047,7 +10064,11 @@
           <t>coder-directive-tasks-part-a.md</t>
         </is>
       </c>
-      <c r="G281" s="11" t="inlineStr"/>
+      <c r="G281" s="11" t="inlineStr">
+        <is>
+          <t>467215f</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="11" t="inlineStr">
@@ -10070,9 +10091,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="E282" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E282" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F282" s="11" t="inlineStr">
@@ -10080,7 +10101,11 @@
           <t>coder-directive-tasks-part-a.md</t>
         </is>
       </c>
-      <c r="G282" s="11" t="inlineStr"/>
+      <c r="G282" s="11" t="inlineStr">
+        <is>
+          <t>34def0e</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="11" t="inlineStr">
@@ -10268,9 +10293,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E288" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E288" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F288" s="11" t="inlineStr">
@@ -10278,7 +10303,11 @@
           <t>coral-task-manager.md</t>
         </is>
       </c>
-      <c r="G288" s="11" t="inlineStr"/>
+      <c r="G288" s="11" t="inlineStr">
+        <is>
+          <t>260e29d — resolveDbId verified</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="11" t="inlineStr">
@@ -10367,9 +10396,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E291" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E291" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F291" s="11" t="inlineStr">
@@ -10379,7 +10408,7 @@
       </c>
       <c r="G291" s="11" t="inlineStr">
         <is>
-          <t>Florin amendment</t>
+          <t>de59819</t>
         </is>
       </c>
     </row>
@@ -10404,9 +10433,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E292" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E292" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F292" s="11" t="inlineStr">
@@ -10414,7 +10443,11 @@
           <t>coder-directive-tasks-part-a.md</t>
         </is>
       </c>
-      <c r="G292" s="11" t="inlineStr"/>
+      <c r="G292" s="11" t="inlineStr">
+        <is>
+          <t>de59819</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="11" t="inlineStr">
@@ -10437,9 +10470,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="E293" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E293" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F293" s="11" t="inlineStr">
@@ -10449,7 +10482,7 @@
       </c>
       <c r="G293" s="11" t="inlineStr">
         <is>
-          <t>Finding F1</t>
+          <t>23047fd</t>
         </is>
       </c>
     </row>
@@ -10511,9 +10544,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E295" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E295" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F295" s="11" t="inlineStr">
@@ -10523,7 +10556,7 @@
       </c>
       <c r="G295" s="11" t="inlineStr">
         <is>
-          <t>Scoped hydration required: schemas + index + loadDatabasePages(db-tasks) only</t>
+          <t>d9216da</t>
         </is>
       </c>
     </row>
@@ -10585,9 +10618,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="E297" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E297" s="12" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F297" s="11" t="inlineStr">
@@ -10597,7 +10630,7 @@
       </c>
       <c r="G297" s="11" t="inlineStr">
         <is>
-          <t>FLORIN DECISION — gates DEP-3/4</t>
+          <t>a2dc5ba built unrequested, breached the desktop fence, took DEP-0 which was Florin's call — KEEP OR REVERT?</t>
         </is>
       </c>
     </row>
@@ -10622,9 +10655,9 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E298" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E298" s="12" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F298" s="11" t="inlineStr">
@@ -10634,7 +10667,7 @@
       </c>
       <c r="G298" s="11" t="inlineStr">
         <is>
-          <t>Silent-failure shape</t>
+          <t>a2dc5ba built unrequested, breached the desktop fence, took DEP-0 which was Florin's call — KEEP OR REVERT?</t>
         </is>
       </c>
     </row>
@@ -10659,9 +10692,9 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E299" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E299" s="12" t="inlineStr">
+        <is>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F299" s="11" t="inlineStr">
@@ -10669,7 +10702,11 @@
           <t>coral-task-dependencies.md</t>
         </is>
       </c>
-      <c r="G299" s="11" t="inlineStr"/>
+      <c r="G299" s="11" t="inlineStr">
+        <is>
+          <t>a2dc5ba built unrequested, breached the desktop fence, took DEP-0 which was Florin's call — KEEP OR REVERT?</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="11" t="inlineStr">
@@ -10815,8 +10852,193 @@
         </is>
       </c>
     </row>
+    <row r="304">
+      <c r="A304" s="11" t="inlineStr">
+        <is>
+          <t>TASK-M10</t>
+        </is>
+      </c>
+      <c r="B304" s="11" t="inlineStr">
+        <is>
+          <t>Assign a task to a project from the mobile list (not in the capture path). Picker sourced from the in-memory pageIndex filtered to db-1 — never loads the projects database</t>
+        </is>
+      </c>
+      <c r="C304" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Mobile</t>
+        </is>
+      </c>
+      <c r="D304" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E304" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F304" s="11" t="inlineStr">
+        <is>
+          <t>coder-directive-tasks-part-a.md</t>
+        </is>
+      </c>
+      <c r="G304" s="11" t="inlineStr">
+        <is>
+          <t>Florin 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="11" t="inlineStr">
+        <is>
+          <t>TASK-NO-SUBDOMAIN</t>
+        </is>
+      </c>
+      <c r="B305" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: no subdomain for tasks — route only. Different origin would split cookies/session on every platform and need a 3rd auth-redirect branch, for no gain (iOS already isolates per installed app)</t>
+        </is>
+      </c>
+      <c r="C305" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Mobile</t>
+        </is>
+      </c>
+      <c r="D305" s="17" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E305" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F305" s="11" t="inlineStr">
+        <is>
+          <t>coral-task-manager.md</t>
+        </is>
+      </c>
+      <c r="G305" s="11" t="inlineStr">
+        <is>
+          <t>D2 — recorded so it is not re-litigated</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="11" t="inlineStr">
+        <is>
+          <t>TASK-A-E1</t>
+        </is>
+      </c>
+      <c r="B306" s="11" t="inlineStr">
+        <is>
+          <t>FLORIN DECISION: keep or revert a2dc5ba (DependencyGraph +283/-60 — desktop fence breach + DEP-0 decided by the coder)</t>
+        </is>
+      </c>
+      <c r="C306" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Process</t>
+        </is>
+      </c>
+      <c r="D306" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E306" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F306" s="11" t="inlineStr">
+        <is>
+          <t>coder-directive-tasks-part-a.md</t>
+        </is>
+      </c>
+      <c r="G306" s="11" t="inlineStr">
+        <is>
+          <t>Plan review 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="11" t="inlineStr">
+        <is>
+          <t>TASK-A-E3</t>
+        </is>
+      </c>
+      <c r="B307" s="11" t="inlineStr">
+        <is>
+          <t>Report the t- vs opt- live count. No hedge: opt-* only, or STOP as PROJ-2 work</t>
+        </is>
+      </c>
+      <c r="C307" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Schema</t>
+        </is>
+      </c>
+      <c r="D307" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E307" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F307" s="11" t="inlineStr">
+        <is>
+          <t>coder-directive-tasks-part-a.md</t>
+        </is>
+      </c>
+      <c r="G307" s="11" t="inlineStr">
+        <is>
+          <t>Plan review 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="11" t="inlineStr">
+        <is>
+          <t>TASK-A-E7</t>
+        </is>
+      </c>
+      <c r="B308" s="11" t="inlineStr">
+        <is>
+          <t>Report measured capture times: 1 tap from the Tasks icon, &lt;=2 taps / &lt;=5s from cold</t>
+        </is>
+      </c>
+      <c r="C308" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Mobile</t>
+        </is>
+      </c>
+      <c r="D308" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E308" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F308" s="11" t="inlineStr">
+        <is>
+          <t>coder-directive-tasks-part-a.md</t>
+        </is>
+      </c>
+      <c r="G308" s="11" t="inlineStr">
+        <is>
+          <t>Plan review 2026-09-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G303"/>
+  <autoFilter ref="A1:G308"/>
   <dataValidations count="1">
     <dataValidation sqref="E2:E203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Done,Blocked,Dropped"</formula1>
@@ -10832,7 +11054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11190,6 +11412,28 @@
       <c r="D16" s="11" t="inlineStr">
         <is>
           <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>TASK-A-E1</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>DECIDE: keep a2dc5ba (dependency engine, built unrequested on a frozen desktop file) or revert it to Part C</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
     </row>
@@ -11236,7 +11480,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>COUNTA(Roadmap!A2:A303)</f>
+        <f>COUNTA(Roadmap!A2:A308)</f>
         <v/>
       </c>
     </row>
@@ -11247,7 +11491,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>COUNTIF(Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIF(Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11258,7 +11502,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTIF(Roadmap!E2:E303,"In progress")</f>
+        <f>COUNTIF(Roadmap!E2:E308,"In progress")</f>
         <v/>
       </c>
     </row>
@@ -11269,7 +11513,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>COUNTIF(Roadmap!E2:E303,"Done")</f>
+        <f>COUNTIF(Roadmap!E2:E308,"Done")</f>
         <v/>
       </c>
     </row>
@@ -11284,7 +11528,7 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>COUNTIF(Roadmap!D2:D303,"P0")</f>
+        <f>COUNTIF(Roadmap!D2:D308,"P0")</f>
         <v/>
       </c>
     </row>
@@ -11295,7 +11539,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>COUNTIFS(Roadmap!D2:D303,"P0",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D308,"P0",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11306,7 +11550,7 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <f>COUNTIF(Roadmap!D2:D303,"P1")</f>
+        <f>COUNTIF(Roadmap!D2:D308,"P1")</f>
         <v/>
       </c>
     </row>
@@ -11317,7 +11561,7 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>COUNTIFS(Roadmap!D2:D303,"P1",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D308,"P1",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11328,7 +11572,7 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>COUNTIF(Roadmap!D2:D303,"P2")</f>
+        <f>COUNTIF(Roadmap!D2:D308,"P2")</f>
         <v/>
       </c>
     </row>
@@ -11339,7 +11583,7 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>COUNTIFS(Roadmap!D2:D303,"P2",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D308,"P2",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11350,7 +11594,7 @@
         </is>
       </c>
       <c r="B13" s="3">
-        <f>COUNTIF(Roadmap!D2:D303,"P3")</f>
+        <f>COUNTIF(Roadmap!D2:D308,"P3")</f>
         <v/>
       </c>
     </row>
@@ -11361,7 +11605,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>COUNTIFS(Roadmap!D2:D303,"P3",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D308,"P3",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11372,7 +11616,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>COUNTIF(Roadmap!D2:D303,"P4")</f>
+        <f>COUNTIF(Roadmap!D2:D308,"P4")</f>
         <v/>
       </c>
     </row>
@@ -11383,7 +11627,7 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <f>COUNTIFS(Roadmap!D2:D303,"P4",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D308,"P4",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11406,7 +11650,7 @@
         </is>
       </c>
       <c r="B19" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Automations",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Automations",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11417,7 +11661,7 @@
         </is>
       </c>
       <c r="B20" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Calendar",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Calendar",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11428,7 +11672,7 @@
         </is>
       </c>
       <c r="B21" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Email attachments",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Email attachments",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11439,7 +11683,7 @@
         </is>
       </c>
       <c r="B22" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Engine · Grid",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Engine · Grid",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11450,7 +11694,7 @@
         </is>
       </c>
       <c r="B23" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Engine · Relations",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Engine · Relations",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11461,7 +11705,7 @@
         </is>
       </c>
       <c r="B24" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Finance · Invoice protest",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Finance · Invoice protest",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11472,7 +11716,7 @@
         </is>
       </c>
       <c r="B25" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Finance · Purchase invoices",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Finance · Purchase invoices",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11483,7 +11727,7 @@
         </is>
       </c>
       <c r="B26" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Finance · Purchase orders",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Finance · Purchase orders",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11494,7 +11738,7 @@
         </is>
       </c>
       <c r="B27" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"HR · Timesheet reporting",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"HR · Timesheet reporting",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11505,7 +11749,7 @@
         </is>
       </c>
       <c r="B28" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"HR · Timesheets page",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"HR · Timesheets page",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11516,7 +11760,7 @@
         </is>
       </c>
       <c r="B29" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Mobile",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Mobile",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11527,7 +11771,7 @@
         </is>
       </c>
       <c r="B30" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Mobile / PWA",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Mobile / PWA",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11538,7 +11782,7 @@
         </is>
       </c>
       <c r="B31" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Performance · Memory",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Performance · Memory",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11549,7 +11793,7 @@
         </is>
       </c>
       <c r="B32" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Pro Hardening",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Pro Hardening",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11560,7 +11804,7 @@
         </is>
       </c>
       <c r="B33" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Projects",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Projects",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11571,7 +11815,7 @@
         </is>
       </c>
       <c r="B34" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Reliability",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Reliability",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11582,7 +11826,7 @@
         </is>
       </c>
       <c r="B35" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Scan · Receipt bulk",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Scan · Receipt bulk",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11593,7 +11837,7 @@
         </is>
       </c>
       <c r="B36" s="3">
-        <f>COUNTIFS(Roadmap!C2:C303,"Triage / core",Roadmap!E2:E303,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C308,"Triage / core",Roadmap!E2:E308,"Open")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(workflows): update execution order, roadmaps, directives, and status specs
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$G$308</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$G$325</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Florin - my actions'!$A$1:$D$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary'!$A$1:$B$36</definedName>
   </definedNames>
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G308"/>
+  <dimension ref="A1:G325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>CANONICAL RESOLVED (Planner verified in DatabaseClone.tsx, 2026-07-26): the tasks property is prop-task-status (name "Status") with options t-todo / t-prog ("Busy") / t-done ("Done"). The opt-to-do / opt-in-prog / opt-done / opt-hold set belongs to a DIFFERENT property, prop-execution-status ("Ex...</t>
+          <t>TASK-STATUS-CONSISTENCY — TWO LIVE SUBSYSTEMS (project t-* vs module opt-*), each with its own writers and automations. NOT drifted data. Unifying means moving creation paths, toggle, progress automation, quote-service, cockpit, detail view, declared options AND data together</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>PARKED by Florin 2026-09-12 for the big project work. db-tasks carve-out only, inside Part A F1</t>
+          <t>PARKED — scope corrected 2026-09-12, see coral-task-status-two-subsystems.md</t>
         </is>
       </c>
     </row>
@@ -8042,7 +8042,7 @@
       </c>
       <c r="G225" s="11" t="inlineStr">
         <is>
-          <t>Backfill source: getBaseDbId(id) — exact, already exists</t>
+          <t>[P3.2] Backfill source: getBaseDbId(id) — exact, already exists</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="G226" s="11" t="inlineStr">
         <is>
-          <t>Was: denormalise tenantId column — WITHDRAWN</t>
+          <t>[P3.3] Was: denormalise tenantId column — WITHDRAWN</t>
         </is>
       </c>
     </row>
@@ -8116,7 +8116,7 @@
       </c>
       <c r="G227" s="11" t="inlineStr">
         <is>
-          <t>Revised after Florin review 2026-09-12</t>
+          <t>[P3.4] Revised after Florin review 2026-09-12</t>
         </is>
       </c>
     </row>
@@ -8153,7 +8153,7 @@
       </c>
       <c r="G228" s="11" t="inlineStr">
         <is>
-          <t>Revised after Florin review 2026-09-12</t>
+          <t>[P3.5] Revised after Florin review 2026-09-12</t>
         </is>
       </c>
     </row>
@@ -8190,7 +8190,7 @@
       </c>
       <c r="G229" s="11" t="inlineStr">
         <is>
-          <t>Revised after Florin review 2026-09-12</t>
+          <t>[P3.5] Revised after Florin review 2026-09-12</t>
         </is>
       </c>
     </row>
@@ -8227,7 +8227,7 @@
       </c>
       <c r="G230" s="11" t="inlineStr">
         <is>
-          <t>Revised after Florin review 2026-09-12</t>
+          <t>[P3.6] Revised after Florin review 2026-09-12</t>
         </is>
       </c>
     </row>
@@ -8264,7 +8264,7 @@
       </c>
       <c r="G231" s="11" t="inlineStr">
         <is>
-          <t>Written first</t>
+          <t>[P4.1] Written first</t>
         </is>
       </c>
     </row>
@@ -8299,7 +8299,11 @@
           <t>coral-r2-write-path.md</t>
         </is>
       </c>
-      <c r="G232" s="11" t="inlineStr"/>
+      <c r="G232" s="11" t="inlineStr">
+        <is>
+          <t>[P4.2]</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="11" t="inlineStr">
@@ -8332,7 +8336,11 @@
           <t>coral-r2-write-path.md</t>
         </is>
       </c>
-      <c r="G233" s="11" t="inlineStr"/>
+      <c r="G233" s="11" t="inlineStr">
+        <is>
+          <t>[P4.3]</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="11" t="inlineStr">
@@ -8365,7 +8373,11 @@
           <t>coral-r2-write-path.md</t>
         </is>
       </c>
-      <c r="G234" s="11" t="inlineStr"/>
+      <c r="G234" s="11" t="inlineStr">
+        <is>
+          <t>[P4.4]</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="11" t="inlineStr">
@@ -8375,7 +8387,7 @@
       </c>
       <c r="B235" s="11" t="inlineStr">
         <is>
-          <t>Split the 2,215-line store into cache / sync / undo / persistence. Behaviourally invisible</t>
+          <t>RE-CUT by R2-6(c): shrink the store to INDEX + WORKING SET + sync queue. NOT a four-way split. Page cache goes; dirty-page protection untouchable</t>
         </is>
       </c>
       <c r="C235" s="11" t="inlineStr">
@@ -8400,7 +8412,7 @@
       </c>
       <c r="G235" s="11" t="inlineStr">
         <is>
-          <t>Last in R2</t>
+          <t>[P4.5] Unblocked</t>
         </is>
       </c>
     </row>
@@ -9453,7 +9465,7 @@
       </c>
       <c r="G264" s="11" t="inlineStr">
         <is>
-          <t>NEW FINDING 2026-09-12</t>
+          <t>[P3.1] NEW FINDING 2026-09-12</t>
         </is>
       </c>
     </row>
@@ -9815,7 +9827,7 @@
       </c>
       <c r="G274" s="11" t="inlineStr">
         <is>
-          <t>Landmine found 2026-09-12</t>
+          <t>[P4.2] Landmine found 2026-09-12</t>
         </is>
       </c>
     </row>
@@ -9877,9 +9889,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E276" s="20" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E276" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F276" s="11" t="inlineStr">
@@ -9889,7 +9901,7 @@
       </c>
       <c r="G276" s="11" t="inlineStr">
         <is>
-          <t>260e29d — ownership filter + opt-* status still to correct</t>
+          <t>66ef43a</t>
         </is>
       </c>
     </row>
@@ -10618,9 +10630,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="E297" s="12" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="E297" s="15" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="F297" s="11" t="inlineStr">
@@ -10630,7 +10642,7 @@
       </c>
       <c r="G297" s="11" t="inlineStr">
         <is>
-          <t>a2dc5ba built unrequested, breached the desktop fence, took DEP-0 which was Florin's call — KEEP OR REVERT?</t>
+          <t>WITHDRAWN 2026-09-12 — Florin: subtasks over dependencies. Feature deleted; stored data left intact</t>
         </is>
       </c>
     </row>
@@ -10655,9 +10667,9 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E298" s="12" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="E298" s="15" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="F298" s="11" t="inlineStr">
@@ -10667,7 +10679,7 @@
       </c>
       <c r="G298" s="11" t="inlineStr">
         <is>
-          <t>a2dc5ba built unrequested, breached the desktop fence, took DEP-0 which was Florin's call — KEEP OR REVERT?</t>
+          <t>WITHDRAWN 2026-09-12 — Florin: subtasks over dependencies. Feature deleted; stored data left intact</t>
         </is>
       </c>
     </row>
@@ -10692,9 +10704,9 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E299" s="12" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="E299" s="15" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="F299" s="11" t="inlineStr">
@@ -10704,7 +10716,7 @@
       </c>
       <c r="G299" s="11" t="inlineStr">
         <is>
-          <t>a2dc5ba built unrequested, breached the desktop fence, took DEP-0 which was Florin's call — KEEP OR REVERT?</t>
+          <t>WITHDRAWN 2026-09-12 — Florin: subtasks over dependencies. Feature deleted; stored data left intact</t>
         </is>
       </c>
     </row>
@@ -10729,9 +10741,9 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E300" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E300" s="15" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="F300" s="11" t="inlineStr">
@@ -10741,7 +10753,7 @@
       </c>
       <c r="G300" s="11" t="inlineStr">
         <is>
-          <t>Needs DEP-0</t>
+          <t>WITHDRAWN 2026-09-12 — Florin: subtasks over dependencies. Feature deleted; stored data left intact</t>
         </is>
       </c>
     </row>
@@ -10766,9 +10778,9 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E301" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E301" s="15" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="F301" s="11" t="inlineStr">
@@ -10778,7 +10790,7 @@
       </c>
       <c r="G301" s="11" t="inlineStr">
         <is>
-          <t>Needs DEP-0</t>
+          <t>WITHDRAWN 2026-09-12 — Florin: subtasks over dependencies. Feature deleted; stored data left intact</t>
         </is>
       </c>
     </row>
@@ -10803,9 +10815,9 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="E302" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E302" s="15" t="inlineStr">
+        <is>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="F302" s="11" t="inlineStr">
@@ -10813,7 +10825,11 @@
           <t>coral-task-dependencies.md</t>
         </is>
       </c>
-      <c r="G302" s="11" t="inlineStr"/>
+      <c r="G302" s="11" t="inlineStr">
+        <is>
+          <t>WITHDRAWN 2026-09-12 — Florin: subtasks over dependencies. Feature deleted; stored data left intact</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="11" t="inlineStr">
@@ -10873,9 +10889,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E304" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E304" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F304" s="11" t="inlineStr">
@@ -10885,7 +10901,7 @@
       </c>
       <c r="G304" s="11" t="inlineStr">
         <is>
-          <t>Florin 2026-09-12</t>
+          <t>896f38f</t>
         </is>
       </c>
     </row>
@@ -10947,9 +10963,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E306" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E306" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F306" s="11" t="inlineStr">
@@ -10959,7 +10975,7 @@
       </c>
       <c r="G306" s="11" t="inlineStr">
         <is>
-          <t>Plan review 2026-09-12</t>
+          <t>[P0.1] RESOLVED: remove entirely -&gt; DEP-REMOVE (item 1.0)</t>
         </is>
       </c>
     </row>
@@ -10984,7 +11000,7 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E307" s="11" t="inlineStr">
+      <c r="E307" s="12" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -10996,7 +11012,7 @@
       </c>
       <c r="G307" s="11" t="inlineStr">
         <is>
-          <t>Plan review 2026-09-12</t>
+          <t>38 t-* records found — gate tripped but run continued. See TASK-STATUS-38</t>
         </is>
       </c>
     </row>
@@ -11021,9 +11037,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="E308" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E308" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F308" s="11" t="inlineStr">
@@ -11033,12 +11049,641 @@
       </c>
       <c r="G308" s="11" t="inlineStr">
         <is>
-          <t>Plan review 2026-09-12</t>
+          <t>2.4 report: 1 tap, 1.2s, 35KB</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="11" t="inlineStr">
+        <is>
+          <t>LAZY-1</t>
+        </is>
+      </c>
+      <c r="B309" s="11" t="inlineStr">
+        <is>
+          <t>SWEEP: which surfaces read store pages without requesting them? Table of surface/databases/broken Y-N. REPORT BEFORE FIXING</t>
+        </is>
+      </c>
+      <c r="C309" s="11" t="inlineStr">
+        <is>
+          <t>Performance · Lazy load</t>
+        </is>
+      </c>
+      <c r="D309" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E309" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F309" s="11" t="inlineStr">
+        <is>
+          <t>coral-lazy-load-regression.md</t>
+        </is>
+      </c>
+      <c r="G309" s="11" t="inlineStr">
+        <is>
+          <t>[P1.1] 19 surfaces audited, 16 broken. NOT on main — promotion blocker, not an outage</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="11" t="inlineStr">
+        <is>
+          <t>LAZY-2</t>
+        </is>
+      </c>
+      <c r="B310" s="11" t="inlineStr">
+        <is>
+          <t>Make not-loaded indistinguishable from empty impossible: usePagesOf(dbId) returning {pages,status}; dev warning naming db + caller</t>
+        </is>
+      </c>
+      <c r="C310" s="11" t="inlineStr">
+        <is>
+          <t>Performance · Lazy load</t>
+        </is>
+      </c>
+      <c r="D310" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E310" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F310" s="11" t="inlineStr">
+        <is>
+          <t>coral-lazy-load-regression.md</t>
+        </is>
+      </c>
+      <c r="G310" s="11" t="inlineStr">
+        <is>
+          <t>[P1.2] Step 0: classify A (needs rows) vs B (needs labels only). Class B uses pageIndex, NOT loadDatabasePages</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="11" t="inlineStr">
+        <is>
+          <t>LAZY-3</t>
+        </is>
+      </c>
+      <c r="B311" s="11" t="inlineStr">
+        <is>
+          <t>Fix TaskModuleShell: resolveDbId at 5 sites + request pages. Fence exception granted (live regression)</t>
+        </is>
+      </c>
+      <c r="C311" s="11" t="inlineStr">
+        <is>
+          <t>Performance · Lazy load</t>
+        </is>
+      </c>
+      <c r="D311" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E311" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F311" s="11" t="inlineStr">
+        <is>
+          <t>coral-lazy-load-regression.md</t>
+        </is>
+      </c>
+      <c r="G311" s="11" t="inlineStr">
+        <is>
+          <t>[P1.3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="11" t="inlineStr">
+        <is>
+          <t>LAZY-4</t>
+        </is>
+      </c>
+      <c r="B312" s="11" t="inlineStr">
+        <is>
+          <t>IS_LAZY_DATA_ENABLED defaults ON in every env — MEM-3c specified a flag with the old path one toggle away. Flip default off until LAZY-1 is clean, or delete the flag</t>
+        </is>
+      </c>
+      <c r="C312" s="11" t="inlineStr">
+        <is>
+          <t>Performance · Lazy load</t>
+        </is>
+      </c>
+      <c r="D312" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E312" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F312" s="11" t="inlineStr">
+        <is>
+          <t>coral-lazy-load-regression.md</t>
+        </is>
+      </c>
+      <c r="G312" s="11" t="inlineStr">
+        <is>
+          <t>1830c55 — flag defaulted to false</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="11" t="inlineStr">
+        <is>
+          <t>TASK-M11</t>
+        </is>
+      </c>
+      <c r="B313" s="11" t="inlineStr">
+        <is>
+          <t>Mobile task detail sheet — tap row opens editable detail (due/defer/flag/priority/notes/project/recurrence/status + delete). PLANNER OMISSION</t>
+        </is>
+      </c>
+      <c r="C313" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Mobile</t>
+        </is>
+      </c>
+      <c r="D313" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E313" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F313" s="11" t="inlineStr">
+        <is>
+          <t>coder-directive-tasks-part-a.md</t>
+        </is>
+      </c>
+      <c r="G313" s="11" t="inlineStr">
+        <is>
+          <t>62865a7</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="11" t="inlineStr">
+        <is>
+          <t>R2-6</t>
+        </is>
+      </c>
+      <c r="B314" s="11" t="inlineStr">
+        <is>
+          <t>DECIDE THE READ MODEL: two read models already exist (Zustand full-database store + React Query). Lazy loading is a mitigation, not a model. (a) keep+lazy (b) index + per-view queries (c) stated hybrid</t>
+        </is>
+      </c>
+      <c r="C314" s="11" t="inlineStr">
+        <is>
+          <t>Persistence (R2)</t>
+        </is>
+      </c>
+      <c r="D314" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E314" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F314" s="11" t="inlineStr">
+        <is>
+          <t>coral-r2-write-path.md</t>
+        </is>
+      </c>
+      <c r="G314" s="11" t="inlineStr">
+        <is>
+          <t>[P0.3] DECIDED (c) HYBRID: INDEX offline + WORKING SET offline-complete + rest per-view query. Driver: site visit must survive signal loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="11" t="inlineStr">
+        <is>
+          <t>LAZY-2b</t>
+        </is>
+      </c>
+      <c r="B315" s="11" t="inlineStr">
+        <is>
+          <t>Class B surfaces (pickers, chips, Cmd+K) fixed via pageIndex/useLabelsOf — never by loading db-clients/db-suppliers/db-articles/db-1. UniversalSearch searches the index; deeper = server query</t>
+        </is>
+      </c>
+      <c r="C315" s="11" t="inlineStr">
+        <is>
+          <t>Performance · Lazy load</t>
+        </is>
+      </c>
+      <c r="D315" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E315" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F315" s="11" t="inlineStr">
+        <is>
+          <t>coral-lazy-load-regression.md</t>
+        </is>
+      </c>
+      <c r="G315" s="11" t="inlineStr">
+        <is>
+          <t>[P1.2] Planner correction — would undo MEM-3 otherwise</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="11" t="inlineStr">
+        <is>
+          <t>PROMOTE-GATE</t>
+        </is>
+      </c>
+      <c r="B316" s="11" t="inlineStr">
+        <is>
+          <t>develop -&gt; main: 99 commits, all 4 money paths changed. Plan + gates + staging pass in coral-promotion-plan.md. G-1: Phase 1 MUST be complete or promotion is a downgrade (16 surfaces work in prod today)</t>
+        </is>
+      </c>
+      <c r="C316" s="11" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="D316" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E316" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F316" s="11" t="inlineStr">
+        <is>
+          <t>coral-promotion-plan.md</t>
+        </is>
+      </c>
+      <c r="G316" s="11" t="inlineStr">
+        <is>
+          <t>99 commits behind</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="11" t="inlineStr">
+        <is>
+          <t>DEP-REMOVE</t>
+        </is>
+      </c>
+      <c r="B317" s="11" t="inlineStr">
+        <is>
+          <t>Delete DependencyEngine.ts, DependencyGraph.tsx, task-dependencies.test.ts and the TaskModuleShell render path + depends-on initialisation. Stored data LEFT UNTOUCHED</t>
+        </is>
+      </c>
+      <c r="C317" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Removal</t>
+        </is>
+      </c>
+      <c r="D317" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E317" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F317" s="11" t="inlineStr">
+        <is>
+          <t>coder-directive-dep-removal.md</t>
+        </is>
+      </c>
+      <c r="G317" s="11" t="inlineStr">
+        <is>
+          <t>4679e08</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="11" t="inlineStr">
+        <is>
+          <t>TASK-SUBTASKS</t>
+        </is>
+      </c>
+      <c r="B318" s="11" t="inlineStr">
+        <is>
+          <t>Subtasks (containment: parent task -&gt; steps) — what Florin wants instead of dependencies. UNSCOPED, unauthorised</t>
+        </is>
+      </c>
+      <c r="C318" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Future</t>
+        </is>
+      </c>
+      <c r="D318" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E318" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F318" s="11" t="inlineStr">
+        <is>
+          <t>coral-task-manager.md</t>
+        </is>
+      </c>
+      <c r="G318" s="11" t="inlineStr">
+        <is>
+          <t>Part B/C scoping</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="11" t="inlineStr">
+        <is>
+          <t>PROMOTE-P1</t>
+        </is>
+      </c>
+      <c r="B319" s="11" t="inlineStr">
+        <is>
+          <t>Verify DB state before promoting: prisma migrate status + migrate diff against production. Expect no pending, empty diff</t>
+        </is>
+      </c>
+      <c r="C319" s="11" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="D319" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E319" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F319" s="11" t="inlineStr">
+        <is>
+          <t>coral-promotion-plan.md</t>
+        </is>
+      </c>
+      <c r="G319" s="11" t="inlineStr">
+        <is>
+          <t>Florin runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="11" t="inlineStr">
+        <is>
+          <t>PROMOTE-STAGING</t>
+        </is>
+      </c>
+      <c r="B320" s="11" t="inlineStr">
+        <is>
+          <t>Cut release/2026-09, deploy to staging, run the 9-point pass with real data before main</t>
+        </is>
+      </c>
+      <c r="C320" s="11" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="D320" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E320" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F320" s="11" t="inlineStr">
+        <is>
+          <t>coral-promotion-plan.md</t>
+        </is>
+      </c>
+      <c r="G320" s="11" t="inlineStr">
+        <is>
+          <t>pd.md Rule 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="11" t="inlineStr">
+        <is>
+          <t>I18N-GATE</t>
+        </is>
+      </c>
+      <c r="B321" s="11" t="inlineStr">
+        <is>
+          <t>Fix I18N-MISSING-KEYS before promotion so the test baseline is honestly green</t>
+        </is>
+      </c>
+      <c r="C321" s="11" t="inlineStr">
+        <is>
+          <t>i18n</t>
+        </is>
+      </c>
+      <c r="D321" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E321" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F321" s="11" t="inlineStr">
+        <is>
+          <t>coral-promotion-plan.md</t>
+        </is>
+      </c>
+      <c r="G321" s="11" t="inlineStr">
+        <is>
+          <t>G-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="11" t="inlineStr">
+        <is>
+          <t>R2-7</t>
+        </is>
+      </c>
+      <c r="B322" s="11" t="inlineStr">
+        <is>
+          <t>What defines a WORKING SET (explicit pin? today scheduled shifts? last-opened?) — FLORIN decision, do not infer</t>
+        </is>
+      </c>
+      <c r="C322" s="11" t="inlineStr">
+        <is>
+          <t>Persistence (R2)</t>
+        </is>
+      </c>
+      <c r="D322" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E322" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F322" s="11" t="inlineStr">
+        <is>
+          <t>coral-r2-write-path.md</t>
+        </is>
+      </c>
+      <c r="G322" s="11" t="inlineStr">
+        <is>
+          <t>[P4.6] Comes up in Phase 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="11" t="inlineStr">
+        <is>
+          <t>R2-6-RULE1</t>
+        </is>
+      </c>
+      <c r="B323" s="11" t="inlineStr">
+        <is>
+          <t>Degrade gracefully, do not enumerate: an uncached record offline shows an honest specific state. LAZY-2 status must include offline-unavailable as distinct from loading/error/empty</t>
+        </is>
+      </c>
+      <c r="C323" s="11" t="inlineStr">
+        <is>
+          <t>Persistence (R2)</t>
+        </is>
+      </c>
+      <c r="D323" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E323" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F323" s="11" t="inlineStr">
+        <is>
+          <t>coral-r2-write-path.md</t>
+        </is>
+      </c>
+      <c r="G323" s="11" t="inlineStr">
+        <is>
+          <t>Binding rule from R2-6(c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="11" t="inlineStr">
+        <is>
+          <t>R2-6-RULE2</t>
+        </is>
+      </c>
+      <c r="B324" s="11" t="inlineStr">
+        <is>
+          <t>The tenant must SEE what they carry offline before losing signal — working set visible and where it matters chosen, not a guessed cache</t>
+        </is>
+      </c>
+      <c r="C324" s="11" t="inlineStr">
+        <is>
+          <t>Persistence (R2)</t>
+        </is>
+      </c>
+      <c r="D324" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E324" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F324" s="11" t="inlineStr">
+        <is>
+          <t>coral-r2-write-path.md</t>
+        </is>
+      </c>
+      <c r="G324" s="11" t="inlineStr">
+        <is>
+          <t>Binding rule from R2-6(c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="11" t="inlineStr">
+        <is>
+          <t>TASK-STATUS-38</t>
+        </is>
+      </c>
+      <c r="B325" s="11" t="inlineStr">
+        <is>
+          <t>RETRACTED: the 38 are NOT legacy. All carry a project; t-* is the live project-subsystem convention with 5 active writers and the progress automation keyed to it. Migrating would break project completion</t>
+        </is>
+      </c>
+      <c r="C325" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Schema</t>
+        </is>
+      </c>
+      <c r="D325" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E325" s="15" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+      <c r="F325" s="11" t="inlineStr">
+        <is>
+          <t>task-status-38-records.sql</t>
+        </is>
+      </c>
+      <c r="G325" s="11" t="inlineStr">
+        <is>
+          <t>Count: t-todo 22 / t-prog 11 / t-done 5</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G308"/>
+  <autoFilter ref="A1:G325"/>
   <dataValidations count="1">
     <dataValidation sqref="E2:E203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Done,Blocked,Dropped"</formula1>
@@ -11054,7 +11699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11423,15 +12068,125 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>DECIDE: keep a2dc5ba (dependency engine, built unrequested on a frozen desktop file) or revert it to Part C</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>DECIDED: remove dependencies entirely; subtasks instead</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>R2-6</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: (c) hybrid — site visit must survive signal loss</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>SEQUENCE</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>coral-execution-order.md is now the single binding sequence — overrides every spec ORDER section</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>R2-6</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: (c) hybrid — site visit must survive signal loss</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>PROMOTION</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Read coral-promotion-plan.md §2 — what changes for you on day one, esp. exported records becoming read-only</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>TASK-STATUS-38</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>DO NOT RUN the UPDATE — retracted. Step 1 count was the finding</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -11480,7 +12235,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>COUNTA(Roadmap!A2:A308)</f>
+        <f>COUNTA(Roadmap!A2:A325)</f>
         <v/>
       </c>
     </row>
@@ -11491,7 +12246,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>COUNTIF(Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIF(Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11502,7 +12257,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTIF(Roadmap!E2:E308,"In progress")</f>
+        <f>COUNTIF(Roadmap!E2:E325,"In progress")</f>
         <v/>
       </c>
     </row>
@@ -11513,7 +12268,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>COUNTIF(Roadmap!E2:E308,"Done")</f>
+        <f>COUNTIF(Roadmap!E2:E325,"Done")</f>
         <v/>
       </c>
     </row>
@@ -11528,7 +12283,7 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>COUNTIF(Roadmap!D2:D308,"P0")</f>
+        <f>COUNTIF(Roadmap!D2:D325,"P0")</f>
         <v/>
       </c>
     </row>
@@ -11539,7 +12294,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>COUNTIFS(Roadmap!D2:D308,"P0",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D325,"P0",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11550,7 +12305,7 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <f>COUNTIF(Roadmap!D2:D308,"P1")</f>
+        <f>COUNTIF(Roadmap!D2:D325,"P1")</f>
         <v/>
       </c>
     </row>
@@ -11561,7 +12316,7 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>COUNTIFS(Roadmap!D2:D308,"P1",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D325,"P1",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11572,7 +12327,7 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>COUNTIF(Roadmap!D2:D308,"P2")</f>
+        <f>COUNTIF(Roadmap!D2:D325,"P2")</f>
         <v/>
       </c>
     </row>
@@ -11583,7 +12338,7 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>COUNTIFS(Roadmap!D2:D308,"P2",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D325,"P2",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11594,7 +12349,7 @@
         </is>
       </c>
       <c r="B13" s="3">
-        <f>COUNTIF(Roadmap!D2:D308,"P3")</f>
+        <f>COUNTIF(Roadmap!D2:D325,"P3")</f>
         <v/>
       </c>
     </row>
@@ -11605,7 +12360,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>COUNTIFS(Roadmap!D2:D308,"P3",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D325,"P3",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11616,7 +12371,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>COUNTIF(Roadmap!D2:D308,"P4")</f>
+        <f>COUNTIF(Roadmap!D2:D325,"P4")</f>
         <v/>
       </c>
     </row>
@@ -11627,7 +12382,7 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <f>COUNTIFS(Roadmap!D2:D308,"P4",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D325,"P4",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11650,7 +12405,7 @@
         </is>
       </c>
       <c r="B19" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Automations",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Automations",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11661,7 +12416,7 @@
         </is>
       </c>
       <c r="B20" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Calendar",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Calendar",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11672,7 +12427,7 @@
         </is>
       </c>
       <c r="B21" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Email attachments",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Email attachments",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11683,7 +12438,7 @@
         </is>
       </c>
       <c r="B22" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Engine · Grid",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Engine · Grid",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11694,7 +12449,7 @@
         </is>
       </c>
       <c r="B23" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Engine · Relations",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Engine · Relations",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11705,7 +12460,7 @@
         </is>
       </c>
       <c r="B24" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Finance · Invoice protest",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Finance · Invoice protest",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11716,7 +12471,7 @@
         </is>
       </c>
       <c r="B25" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Finance · Purchase invoices",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Finance · Purchase invoices",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11727,7 +12482,7 @@
         </is>
       </c>
       <c r="B26" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Finance · Purchase orders",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Finance · Purchase orders",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11738,7 +12493,7 @@
         </is>
       </c>
       <c r="B27" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"HR · Timesheet reporting",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"HR · Timesheet reporting",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11749,7 +12504,7 @@
         </is>
       </c>
       <c r="B28" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"HR · Timesheets page",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"HR · Timesheets page",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11760,7 +12515,7 @@
         </is>
       </c>
       <c r="B29" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Mobile",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Mobile",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11771,7 +12526,7 @@
         </is>
       </c>
       <c r="B30" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Mobile / PWA",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Mobile / PWA",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11782,7 +12537,7 @@
         </is>
       </c>
       <c r="B31" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Performance · Memory",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Performance · Memory",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11793,7 +12548,7 @@
         </is>
       </c>
       <c r="B32" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Pro Hardening",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Pro Hardening",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11804,7 +12559,7 @@
         </is>
       </c>
       <c r="B33" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Projects",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Projects",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11815,7 +12570,7 @@
         </is>
       </c>
       <c r="B34" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Reliability",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Reliability",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11826,7 +12581,7 @@
         </is>
       </c>
       <c r="B35" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Scan · Receipt bulk",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Scan · Receipt bulk",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>
@@ -11837,7 +12592,7 @@
         </is>
       </c>
       <c r="B36" s="3">
-        <f>COUNTIFS(Roadmap!C2:C308,"Triage / core",Roadmap!E2:E308,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C325,"Triage / core",Roadmap!E2:E325,"Open")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(tasks): implement sheet directives and subtasks (TASK-M13..M15, TASK-SUBTASKS)
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$G$325</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$G$334</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Florin - my actions'!$A$1:$D$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary'!$A$1:$B$36</definedName>
   </definedNames>
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G325"/>
+  <dimension ref="A1:G334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -908,9 +908,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -918,7 +918,11 @@
           <t>coral-timesheet-reporting.md:30</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>afbf405</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -8412,7 +8416,7 @@
       </c>
       <c r="G235" s="11" t="inlineStr">
         <is>
-          <t>[P4.5] Unblocked</t>
+          <t>[P4.5] Unblocked. ALSO absorbs LAZY-5: the ~15 surfaces migrate once, and IS_LAZY_DATA_ENABLED is deleted here</t>
         </is>
       </c>
     </row>
@@ -10115,7 +10119,7 @@
       </c>
       <c r="G282" s="11" t="inlineStr">
         <is>
-          <t>34def0e</t>
+          <t>34def0e — fixed the app shell 100vh-&gt;100dvh but MISSED the two sheet max-h-[80/85vh]. See TASK-M12</t>
         </is>
       </c>
     </row>
@@ -11111,9 +11115,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E310" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E310" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F310" s="11" t="inlineStr">
@@ -11123,7 +11127,7 @@
       </c>
       <c r="G310" s="11" t="inlineStr">
         <is>
-          <t>[P1.2] Step 0: classify A (needs rows) vs B (needs labels only). Class B uses pageIndex, NOT loadDatabasePages</t>
+          <t>329370a</t>
         </is>
       </c>
     </row>
@@ -11148,9 +11152,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E311" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E311" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F311" s="11" t="inlineStr">
@@ -11160,7 +11164,7 @@
       </c>
       <c r="G311" s="11" t="inlineStr">
         <is>
-          <t>[P1.3]</t>
+          <t>622eb00</t>
         </is>
       </c>
     </row>
@@ -11296,9 +11300,9 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="E315" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E315" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F315" s="11" t="inlineStr">
@@ -11308,7 +11312,7 @@
       </c>
       <c r="G315" s="11" t="inlineStr">
         <is>
-          <t>[P1.2] Planner correction — would undo MEM-3 otherwise</t>
+          <t>329370a — useLabelsOf built</t>
         </is>
       </c>
     </row>
@@ -11394,7 +11398,7 @@
       </c>
       <c r="B318" s="11" t="inlineStr">
         <is>
-          <t>Subtasks (containment: parent task -&gt; steps) — what Florin wants instead of dependencies. UNSCOPED, unauthorised</t>
+          <t>Subtasks: self-relation prop-task-parent, ONE level, inherit project, inline add in sheet, parent shows 3/5. No auto-close (user closes), no cascade delete (promote to top-level)</t>
         </is>
       </c>
       <c r="C318" s="11" t="inlineStr">
@@ -11404,7 +11408,7 @@
       </c>
       <c r="D318" s="14" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E318" s="11" t="inlineStr">
@@ -11414,12 +11418,12 @@
       </c>
       <c r="F318" s="11" t="inlineStr">
         <is>
-          <t>coral-task-manager.md</t>
+          <t>coral-task-subtasks.md</t>
         </is>
       </c>
       <c r="G318" s="11" t="inlineStr">
         <is>
-          <t>Part B/C scoping</t>
+          <t>[P2.10] Replaces dependencies</t>
         </is>
       </c>
     </row>
@@ -11682,8 +11686,341 @@
         </is>
       </c>
     </row>
+    <row r="326">
+      <c r="A326" s="11" t="inlineStr">
+        <is>
+          <t>LAZY-5</t>
+        </is>
+      </c>
+      <c r="B326" s="11" t="inlineStr">
+        <is>
+          <t>CANCELLED — absorbed into R2-4. Migrating the 15 surfaces to make the OLD lazy model work, then again to the hybrid, would touch each twice. They move once, to the hybrid; the flag is DELETED, not re-enabled</t>
+        </is>
+      </c>
+      <c r="C326" s="11" t="inlineStr">
+        <is>
+          <t>Performance · Lazy load</t>
+        </is>
+      </c>
+      <c r="D326" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E326" s="15" t="inlineStr">
+        <is>
+          <t>Dropped</t>
+        </is>
+      </c>
+      <c r="F326" s="11" t="inlineStr">
+        <is>
+          <t>coral-lazy-load-regression.md</t>
+        </is>
+      </c>
+      <c r="G326" s="11" t="inlineStr">
+        <is>
+          <t>Florin caught this 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="11" t="inlineStr">
+        <is>
+          <t>TASK-M12</t>
+        </is>
+      </c>
+      <c r="B327" s="11" t="inlineStr">
+        <is>
+          <t>One BottomSheet primitive: dvh (not vh), overscroll-contain, body scroll lock, fixed footer for Delete. Fixes scroll-under, elastic bounce, unreachable Delete, no vertical scroll — all one root</t>
+        </is>
+      </c>
+      <c r="C327" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Mobile</t>
+        </is>
+      </c>
+      <c r="D327" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E327" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F327" s="11" t="inlineStr">
+        <is>
+          <t>coder-directive-tasks-sheet.md</t>
+        </is>
+      </c>
+      <c r="G327" s="11" t="inlineStr">
+        <is>
+          <t>[P2.6] 3 hand-rolled sheets, none correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="11" t="inlineStr">
+        <is>
+          <t>TASK-M13</t>
+        </is>
+      </c>
+      <c r="B328" s="11" t="inlineStr">
+        <is>
+          <t>File attachment on a task — camera/library, storage.put tenant-scoped, offline-queued, declare prop-task-attachments</t>
+        </is>
+      </c>
+      <c r="C328" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Mobile</t>
+        </is>
+      </c>
+      <c r="D328" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E328" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F328" s="11" t="inlineStr">
+        <is>
+          <t>coder-directive-tasks-sheet.md</t>
+        </is>
+      </c>
+      <c r="G328" s="11" t="inlineStr">
+        <is>
+          <t>[P2.7] Planner omission</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="11" t="inlineStr">
+        <is>
+          <t>TASK-M14</t>
+        </is>
+      </c>
+      <c r="B329" s="11" t="inlineStr">
+        <is>
+          <t>Recurrence anchor must be a VISIBLE PER-TASK SETTING (from due / from completion) — currently implemented but not exposed — plus show the next computed date</t>
+        </is>
+      </c>
+      <c r="C329" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Mobile</t>
+        </is>
+      </c>
+      <c r="D329" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E329" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F329" s="11" t="inlineStr">
+        <is>
+          <t>coder-directive-tasks-sheet.md</t>
+        </is>
+      </c>
+      <c r="G329" s="11" t="inlineStr">
+        <is>
+          <t>[P2.8]</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="11" t="inlineStr">
+        <is>
+          <t>TASK-M15</t>
+        </is>
+      </c>
+      <c r="B330" s="11" t="inlineStr">
+        <is>
+          <t>Reminders = EMAIL DIGEST (decided). Resend, no new infra. SMS is a later channel choice driven by 2FA, not a reminder project</t>
+        </is>
+      </c>
+      <c r="C330" s="11" t="inlineStr">
+        <is>
+          <t>Tasks · Mobile</t>
+        </is>
+      </c>
+      <c r="D330" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E330" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F330" s="11" t="inlineStr">
+        <is>
+          <t>coder-directive-tasks-sheet.md</t>
+        </is>
+      </c>
+      <c r="G330" s="11" t="inlineStr">
+        <is>
+          <t>[P2.9] DECIDED 2026-09-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="11" t="inlineStr">
+        <is>
+          <t>SMS-1</t>
+        </is>
+      </c>
+      <c r="B331" s="11" t="inlineStr">
+        <is>
+          <t>lib/messaging transport module, provider-agnostic, modelled on lib/storage. Nothing outside it imports the provider SDK</t>
+        </is>
+      </c>
+      <c r="C331" s="11" t="inlineStr">
+        <is>
+          <t>Platform · SMS</t>
+        </is>
+      </c>
+      <c r="D331" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E331" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F331" s="11" t="inlineStr">
+        <is>
+          <t>coral-sms-transport.md</t>
+        </is>
+      </c>
+      <c r="G331" s="11" t="inlineStr">
+        <is>
+          <t>2FA drives it, not reminders</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="11" t="inlineStr">
+        <is>
+          <t>SMS-2</t>
+        </is>
+      </c>
+      <c r="B332" s="11" t="inlineStr">
+        <is>
+          <t>2FA over SMS — FLORIN DECISION on scope (who) + mandatory recovery codes + rate limits + SMS-pumping geo-allowlist</t>
+        </is>
+      </c>
+      <c r="C332" s="11" t="inlineStr">
+        <is>
+          <t>Platform · SMS</t>
+        </is>
+      </c>
+      <c r="D332" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E332" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F332" s="11" t="inlineStr">
+        <is>
+          <t>coral-sms-transport.md</t>
+        </is>
+      </c>
+      <c r="G332" s="11" t="inlineStr">
+        <is>
+          <t>FLORIN DECISION</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="11" t="inlineStr">
+        <is>
+          <t>SMS-3</t>
+        </is>
+      </c>
+      <c r="B333" s="11" t="inlineStr">
+        <is>
+          <t>Reminders as a second SMS consumer — per-user channel choice, per-tenant opt-in and cost ceiling</t>
+        </is>
+      </c>
+      <c r="C333" s="11" t="inlineStr">
+        <is>
+          <t>Platform · SMS</t>
+        </is>
+      </c>
+      <c r="D333" s="17" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E333" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F333" s="11" t="inlineStr">
+        <is>
+          <t>coral-sms-transport.md</t>
+        </is>
+      </c>
+      <c r="G333" s="11" t="inlineStr">
+        <is>
+          <t>After SMS-1/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="11" t="inlineStr">
+        <is>
+          <t>SMS-0</t>
+        </is>
+      </c>
+      <c r="B334" s="11" t="inlineStr">
+        <is>
+          <t>Evaluate providers on BE/EU criteria: route quality, BE alphanumeric sender ID, GDPR residency, fraud controls. NOT on price — at our volume the whole thing is under EUR 5/month. Candidates: Sinch, Plivo, smstools.be (Belgian), Twilio. "Sendly" not found — verify the name</t>
+        </is>
+      </c>
+      <c r="C334" s="11" t="inlineStr">
+        <is>
+          <t>Platform · SMS</t>
+        </is>
+      </c>
+      <c r="D334" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E334" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F334" s="11" t="inlineStr">
+        <is>
+          <t>coral-sms-transport.md</t>
+        </is>
+      </c>
+      <c r="G334" s="11" t="inlineStr">
+        <is>
+          <t>FLORIN — an afternoon with a trial. BE rates ~EUR 0.043-0.066/SMS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G325"/>
+  <autoFilter ref="A1:G334"/>
   <dataValidations count="1">
     <dataValidation sqref="E2:E203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Done,Blocked,Dropped"</formula1>
@@ -11699,7 +12036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12189,6 +12526,50 @@
       <c r="D22" s="11" t="inlineStr">
         <is>
           <t>P0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>TASK-M15</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>DECIDED: email digest now; SMS later, driven by 2FA</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>SMS-0</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Evaluate SMS providers on BE/EU criteria (trial to your phone + a crew phone answers most of it)</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
     </row>
@@ -12235,7 +12616,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>COUNTA(Roadmap!A2:A325)</f>
+        <f>COUNTA(Roadmap!A2:A334)</f>
         <v/>
       </c>
     </row>
@@ -12246,7 +12627,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>COUNTIF(Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIF(Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12257,7 +12638,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTIF(Roadmap!E2:E325,"In progress")</f>
+        <f>COUNTIF(Roadmap!E2:E334,"In progress")</f>
         <v/>
       </c>
     </row>
@@ -12268,7 +12649,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>COUNTIF(Roadmap!E2:E325,"Done")</f>
+        <f>COUNTIF(Roadmap!E2:E334,"Done")</f>
         <v/>
       </c>
     </row>
@@ -12283,7 +12664,7 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>COUNTIF(Roadmap!D2:D325,"P0")</f>
+        <f>COUNTIF(Roadmap!D2:D334,"P0")</f>
         <v/>
       </c>
     </row>
@@ -12294,7 +12675,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>COUNTIFS(Roadmap!D2:D325,"P0",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D334,"P0",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12305,7 +12686,7 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <f>COUNTIF(Roadmap!D2:D325,"P1")</f>
+        <f>COUNTIF(Roadmap!D2:D334,"P1")</f>
         <v/>
       </c>
     </row>
@@ -12316,7 +12697,7 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>COUNTIFS(Roadmap!D2:D325,"P1",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D334,"P1",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12327,7 +12708,7 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>COUNTIF(Roadmap!D2:D325,"P2")</f>
+        <f>COUNTIF(Roadmap!D2:D334,"P2")</f>
         <v/>
       </c>
     </row>
@@ -12338,7 +12719,7 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>COUNTIFS(Roadmap!D2:D325,"P2",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D334,"P2",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12349,7 +12730,7 @@
         </is>
       </c>
       <c r="B13" s="3">
-        <f>COUNTIF(Roadmap!D2:D325,"P3")</f>
+        <f>COUNTIF(Roadmap!D2:D334,"P3")</f>
         <v/>
       </c>
     </row>
@@ -12360,7 +12741,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <f>COUNTIFS(Roadmap!D2:D325,"P3",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D334,"P3",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12371,7 +12752,7 @@
         </is>
       </c>
       <c r="B15" s="3">
-        <f>COUNTIF(Roadmap!D2:D325,"P4")</f>
+        <f>COUNTIF(Roadmap!D2:D334,"P4")</f>
         <v/>
       </c>
     </row>
@@ -12382,7 +12763,7 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <f>COUNTIFS(Roadmap!D2:D325,"P4",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!D2:D334,"P4",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12405,7 +12786,7 @@
         </is>
       </c>
       <c r="B19" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Automations",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Automations",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12416,7 +12797,7 @@
         </is>
       </c>
       <c r="B20" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Calendar",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Calendar",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12427,7 +12808,7 @@
         </is>
       </c>
       <c r="B21" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Email attachments",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Email attachments",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12438,7 +12819,7 @@
         </is>
       </c>
       <c r="B22" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Engine · Grid",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Engine · Grid",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12449,7 +12830,7 @@
         </is>
       </c>
       <c r="B23" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Engine · Relations",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Engine · Relations",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12460,7 +12841,7 @@
         </is>
       </c>
       <c r="B24" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Finance · Invoice protest",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Finance · Invoice protest",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12471,7 +12852,7 @@
         </is>
       </c>
       <c r="B25" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Finance · Purchase invoices",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Finance · Purchase invoices",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12482,7 +12863,7 @@
         </is>
       </c>
       <c r="B26" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Finance · Purchase orders",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Finance · Purchase orders",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12493,7 +12874,7 @@
         </is>
       </c>
       <c r="B27" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"HR · Timesheet reporting",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"HR · Timesheet reporting",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12504,7 +12885,7 @@
         </is>
       </c>
       <c r="B28" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"HR · Timesheets page",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"HR · Timesheets page",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12515,7 +12896,7 @@
         </is>
       </c>
       <c r="B29" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Mobile",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Mobile",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12526,7 +12907,7 @@
         </is>
       </c>
       <c r="B30" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Mobile / PWA",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Mobile / PWA",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12537,7 +12918,7 @@
         </is>
       </c>
       <c r="B31" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Performance · Memory",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Performance · Memory",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12548,7 +12929,7 @@
         </is>
       </c>
       <c r="B32" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Pro Hardening",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Pro Hardening",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12559,7 +12940,7 @@
         </is>
       </c>
       <c r="B33" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Projects",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Projects",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12570,7 +12951,7 @@
         </is>
       </c>
       <c r="B34" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Reliability",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Reliability",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12581,7 +12962,7 @@
         </is>
       </c>
       <c r="B35" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Scan · Receipt bulk",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Scan · Receipt bulk",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>
@@ -12592,7 +12973,7 @@
         </is>
       </c>
       <c r="B36" s="3">
-        <f>COUNTIFS(Roadmap!C2:C325,"Triage / core",Roadmap!E2:E325,"Open")</f>
+        <f>COUNTIFS(Roadmap!C2:C334,"Triage / core",Roadmap!E2:E334,"Open")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(tasks): first-class subtasks on every surface desktop and mobile (coral-task-subtasks)
</commit_message>
<xml_diff>
--- a/.agents/coral-roadmap.xlsx
+++ b/.agents/coral-roadmap.xlsx
@@ -11398,7 +11398,7 @@
       </c>
       <c r="B318" s="11" t="inlineStr">
         <is>
-          <t>Subtasks: self-relation prop-task-parent, ONE level, inherit project, inline add in sheet, parent shows 3/5. No auto-close (user closes), no cascade delete (promote to top-level)</t>
+          <t>Subtasks FIRST-CLASS ON EVERY SURFACE (mobile + desktop list/board/row/review/perspectives + project task tab). Shared lib/tasks/subtasks.ts; no surface recomputes. Child stores NO project — derives from parent, which keeps cockpit/automation/bordereau/po untouched</t>
         </is>
       </c>
       <c r="C318" s="11" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="G318" s="11" t="inlineStr">
         <is>
-          <t>[P2.10] Replaces dependencies</t>
+          <t>[P2.10] REWRITTEN 2026-09-12 — fence lifted for 6 named files + ProjectDetailView task tab</t>
         </is>
       </c>
     </row>
@@ -11879,7 +11879,7 @@
       </c>
       <c r="B331" s="11" t="inlineStr">
         <is>
-          <t>lib/messaging transport module, provider-agnostic, modelled on lib/storage. Nothing outside it imports the provider SDK</t>
+          <t>lib/messaging MessagingProvider implemented against Sweego. Nothing outside lib/messaging imports the Sweego SDK — swapping stays a one-file change</t>
         </is>
       </c>
       <c r="C331" s="11" t="inlineStr">
@@ -11990,7 +11990,7 @@
       </c>
       <c r="B334" s="11" t="inlineStr">
         <is>
-          <t>Evaluate providers on BE/EU criteria: route quality, BE alphanumeric sender ID, GDPR residency, fraud controls. NOT on price — at our volume the whole thing is under EUR 5/month. Candidates: Sinch, Plivo, smstools.be (Belgian), Twilio. "Sendly" not found — verify the name</t>
+          <t>Sweego trial: send to your phone + one crew phone, confirm BE delivery and CORAL sender ID. Check BE price on their worldwide list (EUR 0.040 is the FR price). Credits valid 12 months — buy small</t>
         </is>
       </c>
       <c r="C334" s="11" t="inlineStr">
@@ -12015,7 +12015,7 @@
       </c>
       <c r="G334" s="11" t="inlineStr">
         <is>
-          <t>FLORIN — an afternoon with a trial. BE rates ~EUR 0.043-0.066/SMS</t>
+          <t>DECIDED: Sweego for SMS. Narrowed from evaluation to one confirmation test</t>
         </is>
       </c>
     </row>
@@ -12559,7 +12559,7 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Evaluate SMS providers on BE/EU criteria (trial to your phone + a crew phone answers most of it)</t>
+          <t>Sweego trial: BE delivery + CORAL sender ID to your phone and one crew phone</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">

</xml_diff>